<commit_message>
ajustes en los registros
</commit_message>
<xml_diff>
--- a/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
+++ b/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
@@ -406,13 +406,13 @@
         <v>215569</v>
       </c>
       <c r="D2">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="F2">
         <v>66</v>
       </c>
       <c r="H2">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3">
@@ -425,7 +425,7 @@
         <v>2172.7</v>
       </c>
       <c r="D3">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -541,7 +541,7 @@
         <v>177567</v>
       </c>
       <c r="D9">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="F9">
         <v>34</v>
@@ -639,7 +639,7 @@
         <v>572</v>
       </c>
       <c r="F14">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H14">
         <v>89</v>
@@ -712,7 +712,7 @@
         <v>29658.5</v>
       </c>
       <c r="D18">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F18">
         <v>5</v>
@@ -812,7 +812,7 @@
         <v>152</v>
       </c>
       <c r="F23">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H23">
         <v>29</v>
@@ -831,7 +831,7 @@
         <v>360</v>
       </c>
       <c r="F24">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H24">
         <v>76</v>

</xml_diff>

<commit_message>
mapas de AHO y huella humana
</commit_message>
<xml_diff>
--- a/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
+++ b/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
@@ -406,7 +406,7 @@
         <v>216517</v>
       </c>
       <c r="D2">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="F2">
         <v>66</v>
@@ -428,7 +428,7 @@
         <v>32</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H3">
         <v>5</v>
@@ -539,10 +539,10 @@
         <v>178347</v>
       </c>
       <c r="D9">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="F9">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H9">
         <v>28</v>
@@ -561,7 +561,7 @@
         <v>440</v>
       </c>
       <c r="F10">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H10">
         <v>75</v>
@@ -580,7 +580,7 @@
         <v>116</v>
       </c>
       <c r="F11">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H11">
         <v>19</v>
@@ -634,10 +634,10 @@
         <v>354288</v>
       </c>
       <c r="D14">
-        <v>572</v>
+        <v>568</v>
       </c>
       <c r="F14">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H14">
         <v>89</v>
@@ -726,16 +726,16 @@
         </is>
       </c>
       <c r="B19">
-        <v>16703.4</v>
+        <v>171882</v>
       </c>
       <c r="D19">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F19">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H19">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
@@ -789,7 +789,7 @@
         <v>16</v>
       </c>
       <c r="F22">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H22">
         <v>4</v>
@@ -839,10 +839,8 @@
           <t>Serpocaulon tayronae</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>|EOO cannot be estimated because less than 3 unique pair of coordinates</t>
-        </is>
+      <c r="B25">
+        <v>0.373</v>
       </c>
       <c r="D25">
         <v>8</v>

</xml_diff>

<commit_message>
mapas y scripts actualizados
</commit_message>
<xml_diff>
--- a/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
+++ b/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
@@ -409,7 +409,7 @@
         <v>332</v>
       </c>
       <c r="F2">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H2">
         <v>56</v>
@@ -425,7 +425,7 @@
         <v>2182.1</v>
       </c>
       <c r="D3">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -558,10 +558,10 @@
         <v>319959</v>
       </c>
       <c r="D10">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="F10">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H10">
         <v>75</v>
@@ -637,7 +637,7 @@
         <v>568</v>
       </c>
       <c r="F14">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H14">
         <v>89</v>
@@ -710,7 +710,7 @@
         <v>29789.9</v>
       </c>
       <c r="D18">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F18">
         <v>5</v>
@@ -805,7 +805,7 @@
         <v>196810</v>
       </c>
       <c r="D23">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F23">
         <v>33</v>
@@ -827,7 +827,7 @@
         <v>152</v>
       </c>
       <c r="F24">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H24">
         <v>29</v>
@@ -862,10 +862,10 @@
         <v>992143</v>
       </c>
       <c r="D26">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="F26">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H26">
         <v>76</v>

</xml_diff>

<commit_message>
usé la base de datos llamada "Coordenadas_Serpocaulon" y corrí el script actualizado
</commit_message>
<xml_diff>
--- a/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
+++ b/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
@@ -406,10 +406,10 @@
         <v>216517</v>
       </c>
       <c r="D2">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="F2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H2">
         <v>56</v>
@@ -425,13 +425,13 @@
         <v>2182.1</v>
       </c>
       <c r="D3">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H3">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -488,7 +488,7 @@
         <v>2</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -539,10 +539,10 @@
         <v>178347</v>
       </c>
       <c r="D9">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="F9">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H9">
         <v>28</v>
@@ -634,10 +634,10 @@
         <v>354288</v>
       </c>
       <c r="D14">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="F14">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H14">
         <v>89</v>
@@ -716,7 +716,7 @@
         <v>5</v>
       </c>
       <c r="H18">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19">
@@ -751,7 +751,7 @@
         <v>80</v>
       </c>
       <c r="F20">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H20">
         <v>17</v>
@@ -770,7 +770,7 @@
         <v>28</v>
       </c>
       <c r="F21">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H21">
         <v>5</v>
@@ -789,7 +789,7 @@
         <v>16</v>
       </c>
       <c r="F22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H22">
         <v>4</v>
@@ -805,7 +805,7 @@
         <v>196810</v>
       </c>
       <c r="D23">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F23">
         <v>33</v>
@@ -827,7 +827,7 @@
         <v>152</v>
       </c>
       <c r="F24">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H24">
         <v>29</v>
@@ -849,7 +849,7 @@
         <v>1</v>
       </c>
       <c r="H25">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
@@ -862,7 +862,7 @@
         <v>992143</v>
       </c>
       <c r="D26">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="F26">
         <v>83</v>

</xml_diff>